<commit_message>
Add 20 roles and publish cumulative 43-role workforce scenario
</commit_message>
<xml_diff>
--- a/workforce-model.xlsx
+++ b/workforce-model.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="总览" sheetId="1" r:id="R3d3a53768e8d4f92"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="岗位测算" sheetId="2" r:id="R1089cc9e4bb5465f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务基线" sheetId="3" r:id="R7e56ffc095424a79"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="200万目标" sheetId="4" r:id="Rd13a1a91aae54dba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="总览" sheetId="1" r:id="Ref48d0b3dd3947e5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="岗位测算" sheetId="2" r:id="Rabd1dcf322b44465"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务基线" sheetId="3" r:id="Rd5ac7391dae84c40"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="200万目标" sheetId="4" r:id="Red19bd4190884b4d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -101,7 +101,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="28">
+  <x:cellXfs count="29">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -174,6 +174,9 @@
       <x:alignment vertical="center"/>
     </x:xf>
     <x:xf numFmtId="201" fontId="7" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="7" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
   </x:cellXfs>
@@ -2959,13 +2962,13 @@
   <x:sheetData>
     <x:row r="2">
       <x:c r="A2" s="16" t="str">
-        <x:v>200 万元人力成本目标</x:v>
+        <x:v>追加 20 岗后的累计 43 岗情景</x:v>
       </x:c>
       <x:c r="B2" s="16"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="4" t="str">
-        <x:v>下列黄色参数是董事长情景演算，不是集团已核实的薪酬或可减岗位。</x:v>
+        <x:v>43 岗是董事长压力测试，不是已经核准的人员名单。黄色参数仍需集团填报。</x:v>
       </x:c>
       <x:c r="B3" s="4"/>
     </x:row>
@@ -3155,6 +3158,77 @@
         <x:v>17</x:v>
       </x:c>
     </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="26" t="str">
+        <x:v>原首年 200 万门槛岗位数</x:v>
+      </x:c>
+      <x:c r="B25" s="27" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="D25" s="4" t="str">
+        <x:v>43 岗占约 300 人的 14.3%。每一岗必须有任务取消或合并证据、服务覆盖签字、真实成本和合法用工路径。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="26" t="str">
+        <x:v>董事长追加压减岗位数</x:v>
+      </x:c>
+      <x:c r="B26" s="27" t="n">
+        <x:v>20</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="26" t="str">
+        <x:v>累计岗位压减情景</x:v>
+      </x:c>
+      <x:c r="B27" s="27" t="n">
+        <x:v>43</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="26" t="str">
+        <x:v>全部生效后的期末编制情景</x:v>
+      </x:c>
+      <x:c r="B28" s="27" t="n">
+        <x:v>257</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="26" t="str">
+        <x:v>首年人力成本减少 情景元</x:v>
+      </x:c>
+      <x:c r="B29" s="28" t="n">
+        <x:f>B27*B6*B7/12</x:f>
+        <x:v>3870000</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="26" t="str">
+        <x:v>首年净现金 情景元</x:v>
+      </x:c>
+      <x:c r="B30" s="28" t="n">
+        <x:f>B29-B8-B9</x:f>
+        <x:v>3270000</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="26" t="str">
+        <x:v>稳定年化人力成本减少 情景元</x:v>
+      </x:c>
+      <x:c r="B31" s="28" t="n">
+        <x:f>B27*B6</x:f>
+        <x:v>5160000</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="26" t="str">
+        <x:v>年度可合并工时门槛</x:v>
+      </x:c>
+      <x:c r="B32" s="28" t="n">
+        <x:f>B27*B10</x:f>
+        <x:v>77400</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>